<commit_message>
Add admin page with user settings
</commit_message>
<xml_diff>
--- a/Team02- User Stories.xlsx
+++ b/Team02- User Stories.xlsx
@@ -1,29 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emanuel Vochitoiu\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{445158E9-0798-4C1C-AB9D-FBE01293B0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="User Stories" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="User Stories"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'User Stories'!$A$1:$F$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'User Stories'!$A$1:$F$15</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="60">
   <si>
     <t>ID</t>
   </si>
@@ -232,22 +226,26 @@
     <t>US-14</t>
   </si>
   <si>
+    <t>User</t>
+  </si>
+  <si>
     <t>Admin</t>
   </si>
   <si>
-    <t>As an admin, I can view platform usage metrics including active users and total positions logged so that I can monitor growth and inform future prioritisation.</t>
-  </si>
-  <si>
-    <t>Admin dashboard shows daily and monthly active users
-Total positions and tickers tracked across the platform
-No personal financial data exposed in admin view
-Access restricted to admin role only</t>
+    <t>As a user, I can view and update my account settings so that I can manage my profile and preferences.</t>
+  </si>
+  <si>
+    <t>User can update their display name and email
+User can change their password (requires current password confirmation)
+Changes are saved and reflected immediately
+No other users' data is accessible from this page</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -259,12 +257,15 @@
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFffffff"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
+      <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="14">
@@ -276,62 +277,62 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1A1A2E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8F8FC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFDECEA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE1F5EE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEEEDFE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE6F1FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFAEEDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFAECE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3E2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEAF3DE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF1EFE8"/>
+        <fgColor rgb="FF1a1a2e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFf8f8fc"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFfdecea"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFe1f5ee"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFffffff"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFeeedfe"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFe6f1fb"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFfaeeda"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFfaece7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFfef3e2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFeaf3de"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFf1efe8"/>
       </patternFill>
     </fill>
   </fills>
@@ -345,16 +346,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFD0D0D0"/>
+        <color rgb="FFd0d0d0"/>
       </left>
       <right style="thin">
-        <color rgb="FFD0D0D0"/>
+        <color rgb="FFd0d0d0"/>
       </right>
       <top style="thin">
-        <color rgb="FFD0D0D0"/>
+        <color rgb="FFd0d0d0"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD0D0D0"/>
+        <color rgb="FFd0d0d0"/>
       </bottom>
       <diagonal/>
     </border>
@@ -362,62 +363,68 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+  <cellXfs count="18">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="11" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="12" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="13" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -428,10 +435,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -469,69 +476,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -555,54 +564,53 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
                 <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="15000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
+                <a:tint val="94000"/>
                 <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
+              <a:shade val="9500"/>
               <a:satMod val="105000"/>
             </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -612,7 +620,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -621,7 +629,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -630,7 +638,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -638,10 +646,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -670,7 +678,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
+                <a:tint val="20000"/>
                 <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
@@ -683,13 +691,12 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
                 <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
+                <a:tint val="80000"/>
                 <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
@@ -707,321 +714,322 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
   <dimension ref="A1:F15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="52" customWidth="1"/>
-    <col min="6" max="6" width="60" customWidth="1"/>
+    <col min="1" max="1" style="16" width="8.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="16" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="16" width="12.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="16" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="17" width="52.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="17" width="60.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="28" customFormat="1" s="1">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="46.5" customFormat="1" s="1">
+      <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="46.5" customFormat="1" s="1">
+      <c r="A3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="46.5" customFormat="1" s="1">
+      <c r="A4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="46.5" customFormat="1" s="1">
+      <c r="A5" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="90" customFormat="1" s="1">
+      <c r="A6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="90" customFormat="1" s="1">
+      <c r="A7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="9" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="90" customFormat="1" s="1">
+      <c r="A8" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="90" customFormat="1" s="1">
+      <c r="A9" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="9" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="90" customFormat="1" s="1">
+      <c r="A10" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="90" customFormat="1" s="1">
+      <c r="A11" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="90" customFormat="1" s="1">
+      <c r="A12" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="6" t="s">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="90" customFormat="1" s="1">
+      <c r="A13" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="90" customFormat="1" s="1">
+      <c r="A14" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="6" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="90" customFormat="1" s="1">
+      <c r="A15" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="D15" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="E15" s="8" t="s">
+      <c r="D15" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="E15" s="9" t="s">
         <v>58</v>
       </c>
+      <c r="F15" s="9" t="s">
+        <v>59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F15" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update User Stories excel
</commit_message>
<xml_diff>
--- a/Team02- User Stories.xlsx
+++ b/Team02- User Stories.xlsx
@@ -1,18 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livemdxac-my.sharepoint.com/personal/ev205_live_mdx_ac_uk/Documents/Documents/__Projects/Bloome-PortfolioManagement/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="17" documentId="11_44B0AF93514F2244B0BF1C8C6DE967DE965E578B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6A58BA3-FC4C-4196-9BA8-0F6F1C4637EB}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="User Stories"/>
+    <sheet name="User Stories" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'User Stories'!$A$1:$F$15</definedName>
   </definedNames>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -97,12 +103,6 @@
     <t>As a returning user, I can see my total portfolio value, daily change, and overall gain or loss on a single dashboard so that I understand my financial position at a glance.</t>
   </si>
   <si>
-    <t>Dashboard shows total current value based on live prices
-Daily change shown in both £/$ and percentage
-Overall unrealised P&amp;L shown per holding and as a total
-Dashboard updates automatically during market hours</t>
-  </si>
-  <si>
     <t>US-05</t>
   </si>
   <si>
@@ -202,12 +202,6 @@
     <t>As a returning user, I can see news articles tagged to the specific stock I am viewing so that research and context are available in one place.</t>
   </si>
   <si>
-    <t>Individual stock detail page includes a news panel
-News panel shows the 5 most recent articles for that ticker
-Articles link out to the original source
-Panel refreshes when the page is loaded</t>
-  </si>
-  <si>
     <t>US-13</t>
   </si>
   <si>
@@ -215,12 +209,6 @@
   </si>
   <si>
     <t>As an investor, I can edit or delete a previously logged transaction so that I can correct mistakes without losing my full history.</t>
-  </si>
-  <si>
-    <t>Edit allows changing quantity, price, and date
-Deleting a transaction recalculates portfolio immediately
-Confirmation prompt shown before delete
-Edit history is not exposed to the user in v1</t>
   </si>
   <si>
     <t>US-14</t>
@@ -240,12 +228,28 @@
 Changes are saved and reflected immediately
 No other users' data is accessible from this page</t>
   </si>
+  <si>
+    <t>Edit allows changing quantity, price, and date
+Deleting a transaction recalculates portfolio immediately
+Confirmation prompt shown before delete</t>
+  </si>
+  <si>
+    <t>Individual stock detail page includes a news panel
+News panel shows recent articles for that ticker
+Articles link out to the original source
+Panel refreshes when the page is loaded</t>
+  </si>
+  <si>
+    <t>Dashboard shows total current value based on live prices
+Daily change shown in both £ and percentage
+Overall unrealised P&amp;L shown per holding and as a total
+Dashboard updates automatically during market hours</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -257,7 +261,7 @@
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="FFffffff"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -268,7 +272,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -277,62 +281,44 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1a1a2e"/>
+        <fgColor rgb="FF1A1A2E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFf8f8fc"/>
+        <fgColor rgb="FFF8F8FC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFfdecea"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFe1f5ee"/>
+        <fgColor rgb="FFE6F1FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFffffff"/>
+        <fgColor rgb="FFFAECE7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFeeedfe"/>
+        <fgColor rgb="FFFEF3E2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFe6f1fb"/>
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFfaeeda"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFfaece7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFfef3e2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFeaf3de"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFf1efe8"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -346,16 +332,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFd0d0d0"/>
+        <color rgb="FFD0D0D0"/>
       </left>
       <right style="thin">
-        <color rgb="FFd0d0d0"/>
+        <color rgb="FFD0D0D0"/>
       </right>
       <top style="thin">
-        <color rgb="FFd0d0d0"/>
+        <color rgb="FFD0D0D0"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFd0d0d0"/>
+        <color rgb="FFD0D0D0"/>
       </bottom>
       <diagonal/>
     </border>
@@ -363,68 +349,65 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+  <cellXfs count="16">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="11" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="12" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="13" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -435,10 +418,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -476,71 +459,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -568,7 +551,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -591,11 +574,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -604,13 +587,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -620,7 +603,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -629,7 +612,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -638,7 +621,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -646,10 +629,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -714,22 +697,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:F15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="16" width="8.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="16" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="16" width="12.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="16" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="17" width="52.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="17" width="60.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="8" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="60" style="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="28" customFormat="1" s="1">
+    <row r="1" spans="1:6" s="1" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -749,284 +732,284 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="46.5" customFormat="1" s="1">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:6" s="1" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="46.5" customFormat="1" s="1">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:6" s="1" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="13" t="s">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="46.5" customFormat="1" s="1">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:6" s="1" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="46.5" customFormat="1" s="1">
-      <c r="A5" s="7" t="s">
+    <row r="5" spans="1:6" s="1" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="13" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="12" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="90" customFormat="1" s="1">
-      <c r="A6" s="3" t="s">
+      <c r="B6" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="E6" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C7" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="90" customFormat="1" s="1">
-      <c r="A7" s="7" t="s">
+      <c r="D7" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="E7" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="90" customFormat="1" s="1">
-      <c r="A8" s="3" t="s">
+      <c r="C8" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="D8" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="90" customFormat="1" s="1">
-      <c r="A9" s="7" t="s">
+      <c r="C9" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" s="9" t="s">
+      <c r="F9" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="9" t="s">
+    </row>
+    <row r="10" spans="1:6" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="90" customFormat="1" s="1">
-      <c r="A10" s="3" t="s">
-        <v>39</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="6" t="s">
+      <c r="C10" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="6" t="s">
+    </row>
+    <row r="11" spans="1:6" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="14" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="90" customFormat="1" s="1">
-      <c r="A11" s="7" t="s">
+      <c r="B11" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="F11" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" s="8" t="s">
+      <c r="C13" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="90" customFormat="1" s="1">
-      <c r="A12" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="90" customFormat="1" s="1">
-      <c r="A13" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="F13" s="9" t="s">
+      <c r="E14" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="1" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="12" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="90" customFormat="1" s="1">
-      <c r="A14" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F14" s="6" t="s">
+      <c r="D15" s="12" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="90" customFormat="1" s="1">
-      <c r="A15" s="7" t="s">
+      <c r="E15" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="F15" s="13" t="s">
         <v>56</v>
-      </c>
-      <c r="C15" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>